<commit_message>
Before merging out complete chemical data.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/WardsClustering/artifacts/combined_robustness.xlsx
+++ b/results/02_taxa_assemblage/WardsClustering/artifacts/combined_robustness.xlsx
@@ -605,7 +605,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -615,7 +615,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -662,17 +662,17 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -724,12 +724,12 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1215,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1237,12 +1237,12 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I20" t="n">
@@ -1574,17 +1574,17 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I21" t="n">
@@ -1636,12 +1636,12 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -1842,7 +1842,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Uncertain</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -1864,12 +1864,12 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -1926,7 +1926,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I29" t="n">
@@ -2092,12 +2092,12 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -2429,7 +2429,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -2657,7 +2657,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2667,7 +2667,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I40" t="n">
@@ -2719,12 +2719,12 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I42" t="n">
@@ -2828,17 +2828,17 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Uncertain</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -2890,12 +2890,12 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -2982,7 +2982,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I45" t="n">
@@ -3004,12 +3004,12 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -3039,7 +3039,7 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Core</t>
+          <t>Peripheral</t>
         </is>
       </c>
       <c r="I46" t="n">
@@ -3061,12 +3061,12 @@
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvStrong_TaxaWeak</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Strong</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3351,7 +3351,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>EnvStrong_TaxaStrong</t>
+          <t>EnvWeak_TaxaStrong</t>
         </is>
       </c>
     </row>

</xml_diff>